<commit_message>
Added correct naming convention for screenshot file name. Changed WebSite URl to working URL. Updated locators and test data accordingly.
</commit_message>
<xml_diff>
--- a/testdata/LoginData.xlsx
+++ b/testdata/LoginData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SDET with Jatin\Selenium\Selenium Framework\Automation-Assignment\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60665E91-4174-4680-A987-C003E37185DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A90DDF-3E0B-40D4-9489-C44BB875A541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="5280" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
@@ -33,16 +33,16 @@
     <t>password</t>
   </si>
   <si>
-    <t>yejor31268@noihse.com</t>
+    <t>Anantkinlekar18@gmail.com</t>
+  </si>
+  <si>
+    <t>anant</t>
   </si>
   <si>
     <t>Kishor@123</t>
   </si>
   <si>
-    <t>Anantkinlekar18@gmail.com</t>
-  </si>
-  <si>
-    <t>anant</t>
+    <t>videc95111@manupay.com</t>
   </si>
 </sst>
 </file>
@@ -388,27 +388,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{720F4165-2FE5-457A-8710-716A1CEE5DD3}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{5ADD8A3F-6005-49CB-A4FF-A50DEB9A6259}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{5DDDBD1B-7EFB-4295-9FDA-03ECCEFF2465}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{5DDDBD1B-7EFB-4295-9FDA-03ECCEFF2465}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{994CD693-1BBC-4FC1-BC27-369BDEBABA55}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>